<commit_message>
Enhance dataset cleaning and balancing scripts for improved image processing and organization
</commit_message>
<xml_diff>
--- a/training_history.xlsx
+++ b/training_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,6 +509,64 @@
       </c>
       <c r="G3" t="n">
         <v>0.9133</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-16 12:46:51</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-05-16 12:47:27</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0:00:35.895435</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4200</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9214</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.9322</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.7827</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:13:40</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:14:14</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0:00:34.710811</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4199</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9202</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9449</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.7768</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance SoilApp with detailed predictions and confidence metrics
- Added a progress bar to visualize prediction confidence.
- Implemented detailed output for top 3 class predictions and SOC (Soil Organic Carbon) values.
- Introduced rejection logic for low confidence predictions.
- Updated the UI to display additional information about predictions and SOC categories.
- Added a new confusion matrix file for model evaluation.
- Included a new SVM model file for soil classification.
</commit_message>
<xml_diff>
--- a/training_history.xlsx
+++ b/training_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,16 @@
           <t>R2</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Macro F1</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Weighted F1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -481,6 +491,8 @@
       <c r="G2" t="n">
         <v>0.9133</v>
       </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -510,6 +522,8 @@
       <c r="G3" t="n">
         <v>0.9133</v>
       </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -539,6 +553,8 @@
       <c r="G4" t="n">
         <v>0.7827</v>
       </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -567,6 +583,132 @@
       </c>
       <c r="G5" t="n">
         <v>0.7768</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-20 16:19:17</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-05-20 16:19:55</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0:00:37.729667</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4199</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.9202</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.9449</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.7768</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-20 16:24:35</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-05-20 16:25:10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0:00:34.489773</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4186</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.9296</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>0.9294</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.9295</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-20 16:27:08</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-05-20 16:27:41</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0:00:33.285222</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4186</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.9296</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>0.9294</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.9294</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:45:58</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:46:32</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0:00:33.919578</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4186</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.9356</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>0.9352</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.9353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>